<commit_message>
added START, UPDATE, and VIEW functions
</commit_message>
<xml_diff>
--- a/route_sheet.xlsx
+++ b/route_sheet.xlsx
@@ -8,38 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eriqu\OneDrive\Documents\coding\sms-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CB9F1A7-78EC-4911-99E4-63FBEB837779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE85040-0DC2-468E-A423-6587A2E49860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FA356074-B425-455A-B16B-491C065A7AED}"/>
+    <workbookView xWindow="3420" yWindow="3420" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+  <si>
+    <t>Route number</t>
+  </si>
   <si>
     <t>Start Location</t>
   </si>
@@ -50,15 +34,44 @@
     <t>Destination</t>
   </si>
   <si>
-    <t>Route number</t>
+    <t>status</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>1234 boob dr E</t>
+  </si>
+  <si>
+    <t>4321 penis st</t>
+  </si>
+  <si>
+    <t>Delivered</t>
+  </si>
+  <si>
+    <t>123 tr e</t>
+  </si>
+  <si>
+    <t>In Transit</t>
+  </si>
+  <si>
+    <t>333 poop st</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -86,8 +99,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,8 +435,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C862AB87-0A30-4278-B199-EC91EE285C30}">
-  <dimension ref="A1:D1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -431,18 +445,72 @@
     <col min="4" max="4" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>